<commit_message>
Refactor dashboard and calling list features for improved usability and data handling
- Deleted temporary Excel file related to NQ and NI reasons.
- Updated Dashboard class to include navigation group, label, title, and sort order.
- Enhanced CallingListForm to replace cadence input with a searchable relationship select.
- Modified CallingListsTable to display cadence name and additional lead metrics.
- Improved Workspace component to manage scoreboard presets and display metrics.
- Refactored compliance services to enhance lead dialing logic and cadence handling.
- Updated seeder files to ensure proper cadence associations for calling lists.
- Enhanced tests to verify new scoreboard functionality and agent workspace behavior.
</commit_message>
<xml_diff>
--- a/Docs/NQ and NI Reasons.xlsx
+++ b/Docs/NQ and NI Reasons.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\sf\OnPointCall\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F954D337-E6F8-4D46-8422-8E9E52D96A39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{780ECBA0-2803-4CC3-905E-91265331D034}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38510" yWindow="-110" windowWidth="38620" windowHeight="21220" xr2:uid="{19964D11-EFD9-489F-8D40-5B5181DE269A}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21220" xr2:uid="{19964D11-EFD9-489F-8D40-5B5181DE269A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,53 +39,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="20">
   <si>
     <t>Primary Disposition</t>
   </si>
   <si>
-    <t>What It Means</t>
-  </si>
-  <si>
-    <t>Below minimum age</t>
-  </si>
-  <si>
-    <t>Above maximum age, if applicable</t>
-  </si>
-  <si>
-    <t>Household income below requirement</t>
-  </si>
-  <si>
-    <t>Does not meet credit requirement</t>
-  </si>
-  <si>
-    <t>Spouse/partner required but unavailable</t>
-  </si>
-  <si>
-    <t>Relationship status doesn't meet program criteria</t>
-  </si>
-  <si>
-    <t>Outside required travel radius</t>
-  </si>
-  <si>
-    <t>Existing timeshare ownership issue</t>
-  </si>
-  <si>
-    <t>Homeownership requirement not met</t>
-  </si>
-  <si>
-    <t>Toured too recently</t>
-  </si>
-  <si>
-    <t>Existing/recent package</t>
-  </si>
-  <si>
-    <t>Duplicate lead</t>
-  </si>
-  <si>
-    <t>Doesn't fit predefined categories</t>
-  </si>
-  <si>
     <t>Not Qualified</t>
   </si>
   <si>
@@ -95,68 +53,59 @@
     <t>NQ Credit</t>
   </si>
   <si>
-    <t>Spouse Not Available</t>
-  </si>
-  <si>
-    <t>Single</t>
-  </si>
-  <si>
-    <t>Too Far Away</t>
-  </si>
-  <si>
-    <t>Timeshare Owner</t>
-  </si>
-  <si>
     <t>Not Home Owner</t>
   </si>
   <si>
-    <t>Home Owner less then 3 Years</t>
-  </si>
-  <si>
-    <t>Already toured</t>
-  </si>
-  <si>
-    <t>Already Booked</t>
-  </si>
-  <si>
     <t>Duplicate</t>
   </si>
   <si>
     <t>Other</t>
   </si>
   <si>
-    <t>Below Age</t>
-  </si>
-  <si>
-    <t>Above Age</t>
-  </si>
-  <si>
-    <t>Low Income</t>
-  </si>
-  <si>
-    <t>Single Male</t>
-  </si>
-  <si>
     <t>Too Busy</t>
   </si>
   <si>
     <t>Not Interested</t>
   </si>
   <si>
-    <t>Spouse cannot attend</t>
-  </si>
-  <si>
     <t>Death in Family</t>
   </si>
   <si>
     <t>Reason</t>
+  </si>
+  <si>
+    <t>Income</t>
+  </si>
+  <si>
+    <t>Age</t>
+  </si>
+  <si>
+    <t>Marital Status</t>
+  </si>
+  <si>
+    <t>Travel Club</t>
+  </si>
+  <si>
+    <t>Home Owner Less Then 3 Years</t>
+  </si>
+  <si>
+    <t>Travel Distance</t>
+  </si>
+  <si>
+    <t>Booked</t>
+  </si>
+  <si>
+    <t>Toured</t>
+  </si>
+  <si>
+    <t>Spouse Cannot Attend</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -185,6 +134,12 @@
       <name val="Aptos"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -194,7 +149,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -202,19 +157,36 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -549,215 +521,153 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCD8DA8C-9A1F-4890-BA41-E91EC9913EF3}">
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.1796875" customWidth="1"/>
     <col min="2" max="2" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="95.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C1" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A2" s="1" t="s">
+      <c r="B2" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C2" s="2" t="s">
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A3" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C3" s="2" t="s">
+      <c r="B8" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A10" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A4" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A5" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="A6" s="1" t="s">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A11" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="16" x14ac:dyDescent="0.4">
+      <c r="A12" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A13" s="4"/>
+      <c r="B13" s="4"/>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A14" s="4"/>
+      <c r="B14" s="4"/>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A15" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A16" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A17" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A18" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B18" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A7" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A8" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A9" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A10" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="A11" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C11" s="2"/>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A12" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A13" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A14" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A15" s="1"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A16" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A17" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A20" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="B20" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A21" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="B21" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A22" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="B22" t="s">
-        <v>35</v>
-      </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B15:B18">
+    <sortCondition ref="B15:B18"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>